<commit_message>
Currency conversion: column headings found past a sub-heading row
A uses table with a sub-heading row ("Land Costs", blank across) between its headings
(START, END, METHOD, /RENTABLE SF) and its lines had start and end months merged into one
line and cost per SF named after its method choice. The heading walk now steps over a
sub-heading row, never over an empty row (the edge of the table). r49 carries the
sub-heading rows; the property test reads an amount per SF, per sqm or per kW as money.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016o4U1piqjugt3oSK2Yqgfb
</commit_message>
<xml_diff>
--- a/estatemaster-agent/tests/fixtures/models/r49_retail_dev_usd.xlsx
+++ b/estatemaster-agent/tests/fixtures/models/r49_retail_dev_usd.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="102">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="138" uniqueCount="104">
   <si>
     <t xml:space="preserve">INVESTMENT DESCRIPTION</t>
   </si>
@@ -119,6 +119,9 @@
     <t xml:space="preserve">AMOUNT</t>
   </si>
   <si>
+    <t xml:space="preserve">Land Costs</t>
+  </si>
+  <si>
     <t xml:space="preserve">Land Purchase Price</t>
   </si>
   <si>
@@ -126,6 +129,9 @@
   </si>
   <si>
     <t xml:space="preserve">Closing / Legal Costs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hard Costs</t>
   </si>
   <si>
     <t xml:space="preserve">Site Work</t>
@@ -1683,9 +1689,14 @@
         <v>31</v>
       </c>
     </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B26" s="0" t="s">
+        <v>32</v>
+      </c>
+    </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B27" s="0" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="D27" s="0" t="n">
         <v>0</v>
@@ -1694,7 +1705,7 @@
         <v>0</v>
       </c>
       <c r="F27" s="0" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="H27" s="0" t="n">
         <f aca="false">I27/$E$18</f>
@@ -1706,16 +1717,16 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B28" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="D28" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="E28" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="F28" s="0" t="s">
         <v>34</v>
-      </c>
-      <c r="D28" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="E28" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="F28" s="0" t="s">
-        <v>33</v>
       </c>
       <c r="H28" s="0" t="n">
         <f aca="false">I28/$E$18</f>
@@ -1726,9 +1737,14 @@
         <v>98000</v>
       </c>
     </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B29" s="0" t="s">
+        <v>36</v>
+      </c>
+    </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B30" s="0" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="D30" s="0" t="n">
         <v>2</v>
@@ -1737,7 +1753,7 @@
         <v>8</v>
       </c>
       <c r="F30" s="0" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="H30" s="0" t="n">
         <v>14</v>
@@ -1749,7 +1765,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B31" s="0" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="D31" s="0" t="n">
         <v>4</v>
@@ -1758,7 +1774,7 @@
         <v>16</v>
       </c>
       <c r="F31" s="0" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="H31" s="0" t="n">
         <v>118</v>
@@ -1770,7 +1786,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B32" s="0" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="D32" s="0" t="n">
         <v>12</v>
@@ -1779,7 +1795,7 @@
         <v>20</v>
       </c>
       <c r="F32" s="0" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="H32" s="0" t="n">
         <v>42</v>
@@ -1791,7 +1807,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B33" s="0" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="D33" s="0" t="n">
         <v>1</v>
@@ -1800,7 +1816,7 @@
         <v>20</v>
       </c>
       <c r="F33" s="0" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="H33" s="0" t="n">
         <f aca="false">I33/$E$18</f>
@@ -1813,7 +1829,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B34" s="0" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="D34" s="0" t="n">
         <v>1</v>
@@ -1822,7 +1838,7 @@
         <v>20</v>
       </c>
       <c r="F34" s="0" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="H34" s="0" t="n">
         <f aca="false">I34/$E$18</f>
@@ -1835,7 +1851,7 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B35" s="0" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="D35" s="0" t="n">
         <v>4</v>
@@ -1844,7 +1860,7 @@
         <v>20</v>
       </c>
       <c r="F35" s="0" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="H35" s="0" t="n">
         <f aca="false">I35/$E$18</f>
@@ -1866,7 +1882,7 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B40" s="0" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="E40" s="1" t="n">
         <v>0.6</v>
@@ -1874,7 +1890,7 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B41" s="0" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="E41" s="1" t="n">
         <v>0.0775</v>
@@ -1882,7 +1898,7 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B42" s="0" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="E42" s="1" t="n">
         <v>0.6</v>
@@ -1890,7 +1906,7 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B43" s="0" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E43" s="1" t="n">
         <v>0.0625</v>
@@ -1898,7 +1914,7 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B44" s="0" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="E44" s="0" t="n">
         <v>30</v>
@@ -1906,44 +1922,44 @@
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B91" s="0" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B92" s="0" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="C92" s="0" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="D92" s="0" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="E92" s="0" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="F92" s="0" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="G92" s="0" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="H92" s="0" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="I92" s="0" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="K92" s="0" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B93" s="0" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C93" s="0" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="D93" s="0" t="n">
         <v>18</v>
@@ -1966,15 +1982,15 @@
         <v>1092000</v>
       </c>
       <c r="K93" s="5" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
     </row>
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B94" s="0" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="C94" s="0" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="D94" s="0" t="n">
         <v>20</v>
@@ -1997,15 +2013,15 @@
         <v>147000</v>
       </c>
       <c r="K94" s="5" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B95" s="0" t="s">
+        <v>65</v>
+      </c>
+      <c r="C95" s="0" t="s">
         <v>63</v>
-      </c>
-      <c r="C95" s="0" t="s">
-        <v>61</v>
       </c>
       <c r="D95" s="0" t="n">
         <v>22</v>
@@ -2028,15 +2044,15 @@
         <v>126000</v>
       </c>
       <c r="K95" s="5" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
     </row>
     <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B96" s="0" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="C96" s="0" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="D96" s="0" t="n">
         <v>24</v>
@@ -2059,15 +2075,15 @@
         <v>122400</v>
       </c>
       <c r="K96" s="5" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
     </row>
     <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B97" s="0" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="C97" s="0" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="D97" s="0" t="n">
         <v>26</v>
@@ -2090,15 +2106,15 @@
         <v>103600</v>
       </c>
       <c r="K97" s="5" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
     </row>
     <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B98" s="0" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="C98" s="0" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="D98" s="0" t="n">
         <v>22</v>
@@ -2121,15 +2137,15 @@
         <v>192000</v>
       </c>
       <c r="K98" s="5" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
     </row>
     <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B99" s="0" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="C99" s="0" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="D99" s="0" t="n">
         <v>28</v>
@@ -2152,15 +2168,15 @@
         <v>166400</v>
       </c>
       <c r="K99" s="5" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
     </row>
     <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B100" s="0" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="C100" s="0" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="D100" s="0" t="n">
         <v>16</v>
@@ -2183,15 +2199,15 @@
         <v>185600</v>
       </c>
       <c r="K100" s="5" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
     </row>
     <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B101" s="0" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="C101" s="0" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="D101" s="0" t="n">
         <v>18</v>
@@ -2214,12 +2230,12 @@
         <v>153600</v>
       </c>
       <c r="K101" s="5" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
     </row>
     <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B105" s="0" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="E105" s="0" t="n">
         <f aca="false">SUM(E93:E101)</f>
@@ -2236,7 +2252,7 @@
     </row>
     <row r="120" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B120" s="0" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="E120" s="0" t="n">
         <v>7.4</v>
@@ -2244,7 +2260,7 @@
     </row>
     <row r="121" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B121" s="0" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="E121" s="1" t="n">
         <v>0.03</v>
@@ -2252,7 +2268,7 @@
     </row>
     <row r="122" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B122" s="0" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="E122" s="1" t="n">
         <v>0.9</v>
@@ -2260,7 +2276,7 @@
     </row>
     <row r="123" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B123" s="0" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="E123" s="1" t="n">
         <v>0.05</v>
@@ -2268,7 +2284,7 @@
     </row>
     <row r="124" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B124" s="0" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="E124" s="1" t="n">
         <v>0.07</v>
@@ -2276,7 +2292,7 @@
     </row>
     <row r="125" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B125" s="0" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="E125" s="1" t="n">
         <v>0.02</v>
@@ -2292,7 +2308,7 @@
     </row>
     <row r="130" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B130" s="0" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="E130" s="1" t="n">
         <v>0.9</v>
@@ -2300,7 +2316,7 @@
     </row>
     <row r="131" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B131" s="0" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="E131" s="1" t="n">
         <v>0.08</v>
@@ -2308,7 +2324,7 @@
     </row>
     <row r="132" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B132" s="0" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="E132" s="1" t="n">
         <v>0.2</v>
@@ -2316,7 +2332,7 @@
     </row>
     <row r="140" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B140" s="0" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="L140" s="7" t="n">
         <f aca="false">(L$3&lt;=$I$15)*(((L$3&gt;=$F$93)*$I$93/12*(1+$G$93)^IF($K$93="Annual",INT(MAX(0,L$3-$F$93)/12),5*INT(MAX(0,L$3-$F$93)/60)))+((L$3&gt;=$F$94)*$I$94/12*(1+$G$94)^IF($K$94="Annual",INT(MAX(0,L$3-$F$94)/12),5*INT(MAX(0,L$3-$F$94)/60)))+((L$3&gt;=$F$95)*$I$95/12*(1+$G$95)^IF($K$95="Annual",INT(MAX(0,L$3-$F$95)/12),5*INT(MAX(0,L$3-$F$95)/60)))+((L$3&gt;=$F$96)*$I$96/12*(1+$G$96)^IF($K$96="Annual",INT(MAX(0,L$3-$F$96)/12),5*INT(MAX(0,L$3-$F$96)/60)))+((L$3&gt;=$F$97)*$I$97/12*(1+$G$97)^IF($K$97="Annual",INT(MAX(0,L$3-$F$97)/12),5*INT(MAX(0,L$3-$F$97)/60)))+((L$3&gt;=$F$98)*$I$98/12*(1+$G$98)^IF($K$98="Annual",INT(MAX(0,L$3-$F$98)/12),5*INT(MAX(0,L$3-$F$98)/60)))+((L$3&gt;=$F$99)*$I$99/12*(1+$G$99)^IF($K$99="Annual",INT(MAX(0,L$3-$F$99)/12),5*INT(MAX(0,L$3-$F$99)/60)))+((L$3&gt;=$F$100)*$I$100/12*(1+$G$100)^IF($K$100="Annual",INT(MAX(0,L$3-$F$100)/12),5*INT(MAX(0,L$3-$F$100)/60)))+((L$3&gt;=$F$101)*$I$101/12*(1+$G$101)^IF($K$101="Annual",INT(MAX(0,L$3-$F$101)/12),5*INT(MAX(0,L$3-$F$101)/60))))</f>
@@ -2757,7 +2773,7 @@
     </row>
     <row r="141" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B141" s="0" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="L141" s="7" t="n">
         <f aca="false">L144*$E$122*((L$3&gt;=$F$93)*$E$93+(L$3&gt;=$F$94)*$E$94+(L$3&gt;=$F$95)*$E$95+(L$3&gt;=$F$96)*$E$96+(L$3&gt;=$F$97)*$E$97+(L$3&gt;=$F$98)*$E$98+(L$3&gt;=$F$99)*$E$99+(L$3&gt;=$F$100)*$E$100+(L$3&gt;=$F$101)*$E$101)/$E$105</f>
@@ -3198,7 +3214,7 @@
     </row>
     <row r="142" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B142" s="0" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="L142" s="7" t="n">
         <f aca="false">-$E$123*(L140+L141)</f>
@@ -3639,7 +3655,7 @@
     </row>
     <row r="143" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B143" s="0" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="L143" s="7" t="n">
         <f aca="false">SUM(L140:L142)</f>
@@ -4080,7 +4096,7 @@
     </row>
     <row r="144" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B144" s="0" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="L144" s="7" t="n">
         <f aca="false">(L$3&lt;=$I$15)*(L$3&gt;=MIN($F$93:$F$101))*$E$120*$E$105/12*(1+$E$121)^INT(L$3/12)</f>
@@ -4521,7 +4537,7 @@
     </row>
     <row r="145" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B145" s="0" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="L145" s="7" t="n">
         <f aca="false">L143-L144</f>
@@ -4962,7 +4978,7 @@
     </row>
     <row r="150" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B150" s="0" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="L150" s="7" t="n">
         <f aca="false">IF(AND(L$3&gt;=$D$27,L$3&lt;=$E$27),$I$27*IF($F$27="S-Curve",(COS(PI()*(L$3-$D$27)/($E$27-$D$27+1))-COS(PI()*(L$3-$D$27+1)/($E$27-$D$27+1)))/2,1/($E$27-$D$27+1)),0)+IF(AND(L$3&gt;=$D$28,L$3&lt;=$E$28),$I$28*IF($F$28="S-Curve",(COS(PI()*(L$3-$D$28)/($E$28-$D$28+1))-COS(PI()*(L$3-$D$28+1)/($E$28-$D$28+1)))/2,1/($E$28-$D$28+1)),0)+IF(AND(L$3&gt;=$D$30,L$3&lt;=$E$30),$I$30*IF($F$30="S-Curve",(COS(PI()*(L$3-$D$30)/($E$30-$D$30+1))-COS(PI()*(L$3-$D$30+1)/($E$30-$D$30+1)))/2,1/($E$30-$D$30+1)),0)+IF(AND(L$3&gt;=$D$31,L$3&lt;=$E$31),$I$31*IF($F$31="S-Curve",(COS(PI()*(L$3-$D$31)/($E$31-$D$31+1))-COS(PI()*(L$3-$D$31+1)/($E$31-$D$31+1)))/2,1/($E$31-$D$31+1)),0)+IF(AND(L$3&gt;=$D$32,L$3&lt;=$E$32),$I$32*IF($F$32="S-Curve",(COS(PI()*(L$3-$D$32)/($E$32-$D$32+1))-COS(PI()*(L$3-$D$32+1)/($E$32-$D$32+1)))/2,1/($E$32-$D$32+1)),0)+IF(AND(L$3&gt;=$D$33,L$3&lt;=$E$33),$I$33*IF($F$33="S-Curve",(COS(PI()*(L$3-$D$33)/($E$33-$D$33+1))-COS(PI()*(L$3-$D$33+1)/($E$33-$D$33+1)))/2,1/($E$33-$D$33+1)),0)+IF(AND(L$3&gt;=$D$34,L$3&lt;=$E$34),$I$34*IF($F$34="S-Curve",(COS(PI()*(L$3-$D$34)/($E$34-$D$34+1))-COS(PI()*(L$3-$D$34+1)/($E$34-$D$34+1)))/2,1/($E$34-$D$34+1)),0)+IF(AND(L$3&gt;=$D$35,L$3&lt;=$E$35),$I$35*IF($F$35="S-Curve",(COS(PI()*(L$3-$D$35)/($E$35-$D$35+1))-COS(PI()*(L$3-$D$35+1)/($E$35-$D$35+1)))/2,1/($E$35-$D$35+1)),0)</f>
@@ -5403,7 +5419,7 @@
     </row>
     <row r="151" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B151" s="0" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="L151" s="7" t="n">
         <f aca="false">L150*$E$40</f>
@@ -5844,7 +5860,7 @@
     </row>
     <row r="152" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B152" s="0" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="L152" s="7" t="n">
         <f aca="false">0</f>
@@ -6285,7 +6301,7 @@
     </row>
     <row r="153" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B153" s="0" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="L153" s="7" t="n">
         <f aca="false">0+L151-L154</f>
@@ -6726,7 +6742,7 @@
     </row>
     <row r="154" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B154" s="0" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="L154" s="7" t="n">
         <f aca="false">IF(L$3=$E$44,0+L151,0)</f>
@@ -7167,7 +7183,7 @@
     </row>
     <row r="155" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B155" s="0" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="L155" s="7" t="n">
         <f aca="false">IF(L$3=$E$44,$E$42*12*SUMPRODUCT(($L$3:$DP$3&gt;$E$44)*($L$3:$DP$3&lt;=$E$44+12)*$L$145:$DP$145)/12/$E$126,0)</f>
@@ -7608,7 +7624,7 @@
     </row>
     <row r="156" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B156" s="0" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="L156" s="7" t="n">
         <f aca="false">IF(AND(L$3&gt;$E$44,(L$3&lt;=$I$15)),SUM($L$155:$DP$155)*$E$43/12,0)</f>
@@ -8049,7 +8065,7 @@
     </row>
     <row r="157" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B157" s="0" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="L157" s="7" t="n">
         <f aca="false">IF(L$3=$I$15,SUM($L$155:$DP$155),0)</f>
@@ -8490,7 +8506,7 @@
     </row>
     <row r="160" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B160" s="0" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="L160" s="7" t="n">
         <f aca="false">IF(L$3=$I$15,SUMPRODUCT(($L$3:$DP$3&gt;$I$15-12)*($L$3:$DP$3&lt;=$I$15)*$L$145:$DP$145)*(1+$E$121)/$E$124,0)</f>
@@ -8931,7 +8947,7 @@
     </row>
     <row r="161" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B161" s="0" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="L161" s="7" t="n">
         <f aca="false">-L160*$E$125</f>
@@ -9372,18 +9388,18 @@
     </row>
     <row r="210" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G210" s="0" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="H210" s="0" t="s">
         <v>6</v>
       </c>
       <c r="I210" s="0" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
     </row>
     <row r="211" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B211" s="0" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="G211" s="2" t="n">
         <f aca="false">SUMIF($L$211:$DP$211,"&gt;0")/-SUMIF($L$211:$DP$211,"&lt;0")</f>
@@ -9836,7 +9852,7 @@
     </row>
     <row r="212" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B212" s="0" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="G212" s="2" t="n">
         <f aca="false">SUMIF($L$212:$DP$212,"&gt;0")/-SUMIF($L$212:$DP$212,"&lt;0")</f>
@@ -11222,7 +11238,7 @@
     </row>
     <row r="232" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B232" s="0" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="I232" s="4" t="n">
         <f aca="false">-SUMIF($L$212:$DP$212,"&lt;0")</f>
@@ -11231,7 +11247,7 @@
     </row>
     <row r="233" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B233" s="0" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="I233" s="4" t="n">
         <f aca="false">MAX(0,$E$132*($I$212-$E$131*$I$232*$I$15/12))</f>

</xml_diff>